<commit_message>
Streamline the shared venue sheet to one Venues tab
The Proton Sheet collaborators share now has a single Venues tab with
20 columns in the venue page's order: admin, venue details, freeform
venue notes, one Private notes column (never published, replacing the
four contact columns), and upkeep. Location precision, Verified by and
Submitted by are gone.

The schema moves out of the sheet into tools/find-a-venue/field_guide.csv,
which the sync reads, so exports only need the Venues tab. The newsletter
history, past events and a copy of the Field guide live in a private
reference workbook (data/off_tech_tabs.xlsx).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/find-a-venue/data/off_tech_tabs.xlsx
+++ b/tools/find-a-venue/data/off_tech_tabs.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Off Tech history" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Past events" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field guide" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18981,4 +18982,527 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Shown on site?</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Allowed values</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>What to enter</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Venue ID</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>The venue's web address on the site. Leave blank for a new venue (the sync creates one), and never change it once set.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Approved · Pending review · Archived</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Only Approved venues appear on the site. New venues start as Pending review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Venue name</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Venue details</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Common name of the space.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Venue type</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Venue details</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Park / public space · Privately owned public space (POPS) · Library · Bar / cafe / restaurant · Club / event venue · Arts / community space · Gallery / museum · Bookstore · Church / meeting house · University · Makerspace · Community tech space · Radio station / studio · Other</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>What kind of place this is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Venue details</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Street address, or cross streets for a park. Public places only: never a private home.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Neighborhood</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Venue details</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Borough</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Venue details</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Manhattan · Brooklyn · Queens · Bronx · Staten Island</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Indoor / outdoor</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Venue details</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Indoor · Outdoor · Both</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Capacity (est.)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Venue details</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Rough number of people the space holds. An estimate is fine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Venue details</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Free · Donation · Purchase / minimum spend · Rental fee · Ticketed by venue · Unknown</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Shown as 'Public / cost'. Parks, plazas and libraries also show as public spaces.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>How to book</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Venue notes</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Freeform. Who to ask, how far ahead, permits, any fees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Venue notes</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Freeform and PUBLIC: an events email, booking form or front desk. Never a personal email or phone; put those in Private notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Food &amp; drink</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Venue notes</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Freeform. Outside food OK? Purchase required? Alcohol?</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Venue notes</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Freeform. Step-free entry, elevator, accessible restroom, seating, lighting, quiet corner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>A/V equipment</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Venue notes</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Freeform. Power outlets, sound system or mic, projector or screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Other notes</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Venue notes</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Freeform. Anything else: where to set up, what's worked, what to avoid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Private notes</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Collaborators only</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Never published. Personal contacts (name, email, phone), who knows the venue, anything sensitive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Last verified</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Upkeep</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Date someone last confirmed these details (YYYY-MM-DD).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Latitude</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Upkeep</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Decimal degrees. Leave blank and the sync fills it in from the address.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Longitude</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Upkeep</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Decimal degrees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Copied from tools/find-a-venue/field_guide.csv, which the sync reads. Edit it there.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>